<commit_message>
Planilha da demonstracao vai de 15 para 56 linhas
Em 15 linhas alguem da sala pensa "isso eu fazia na mao em dez minutos",
e a pergunta do momento 1 perde o efeito. O tamanho e metade do argumento
da aula, nao capricho.

Agora sao 14 insumos x 4 fornecedores. O tamanho comprou uma quarta
armadilha, que e a melhor: a Cearapel cota a chapa CTP em caixa com 10 e
os outros por unidade, entao ler o numero direto multiplica o item por
dez. Ninguem acha isso passando o olho em 56 linhas.

O desfecho ficou melhor: sobra um unico fornecedor que cotou os 14 itens
e entrega a tempo, e e o mais caro na conta ingenua. O pedido vago escolhe
o mais barato justamente porque ele esta incompleto.

G13 passa a conferir sete afirmacoes sobre essa planilha, nas duas paginas.
Testado contra copias quebradas: cinco das sete reprovam.

Piso de 50 linhas para insumo virou regra no CLAUDE.md secao 8-ter.
</commit_message>
<xml_diff>
--- a/m1/a1-ecossistema-e-fisica/demonstracao/cotacoes-fornecedores.xlsx
+++ b/m1/a1-ecossistema-e-fisica/demonstracao/cotacoes-fornecedores.xlsx
@@ -442,12 +442,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mapa de cotação · OS 2481 · catálogo institucional 20.000 ex. · exportado em 13/07/2026 14:22</t>
+          <t>Mapa de cotação · OS 2481 · catálogo institucional 20.000 ex. · exportado em 14/07/2026 17:38</t>
         </is>
       </c>
     </row>
@@ -659,11 +659,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Papel offset 90g 66x96</t>
+          <t>Papel couché brilho 150g 66x96</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -672,32 +672,32 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>120</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Papelaria Norte</t>
+          <t>Distribuidora Cearapel</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>172.5</v>
+        <v>276.5</v>
       </c>
       <c r="G8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CIF</t>
+          <t>F.O.B.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>28 dias</t>
+          <t>21 dias</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>14/07/2026</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Papel offset 90g 66x96</t>
+          <t>Papel couché fosco 170g 66x96</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -716,34 +716,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Insumos Delta</t>
+          <t>Papelaria Norte</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>168,00</t>
+          <t>324,00</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>fob</t>
+          <t>CIF</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>45 dias</t>
+          <t>28 dias</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>13-07-26</t>
+          <t>13/07/2026</t>
         </is>
       </c>
     </row>
@@ -753,7 +753,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Papel offset 90g 66x96</t>
+          <t>Papel couché fosco 170g 66x96</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -762,119 +762,122 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Gráfica Suprimentos SA</t>
-        </is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>309.5</v>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>C.I.F.</t>
+          <t>fob</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>à vista (3% desc.)</t>
+          <t>45 dias</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>13-07-26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tinta escala cyan</t>
+          <t>Papel couché fosco 170g 66x96</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>18</v>
+        <v>80</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Papelaria Norte</t>
+          <t>Gráfica Suprimentos SA</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>148</v>
+        <v>318</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CIF</t>
+          <t>C.I.F.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>28 dias</t>
+          <t>à vista (3% desc.)</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Papel couché fosco 170g 66x96</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>80</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>312,00</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
         <v>3</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Tinta escala cyan</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>18</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Insumos Delta</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>139,00</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>12</v>
-      </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>fob</t>
+          <t>F.O.B.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>45 dias</t>
+          <t>21 dias</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>13-07-26</t>
+          <t>14/07/2026</t>
         </is>
       </c>
     </row>
@@ -884,131 +887,170 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Tinta escala cyan</t>
+          <t>Papel offset 90g 66x96</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Gráfica Suprimentos SA</t>
+          <t>Papelaria Norte</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>142.5</v>
+        <v>172.5</v>
       </c>
       <c r="G13" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>C.I.F.</t>
+          <t>CIF</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>à vista (3% desc.)</t>
+          <t>28 dias</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Papel offset 90g 66x96</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>168</v>
+      </c>
+      <c r="G14" t="n">
+        <v>12</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verniz UV brilho</t>
+          <t>Papel offset 90g 66x96</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>litro</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Papelaria Norte</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>96,00</t>
+          <t>Gráfica Suprimentos SA</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>CIF</t>
+          <t>C.I.F.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>28 dias</t>
+          <t>à vista (3% desc.)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verniz UV brilho</t>
+          <t>Papel offset 90g 66x96</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>litro</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Insumos Delta</t>
+          <t>Distribuidora Cearapel</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>91</v>
+        <v>170</v>
       </c>
       <c r="G16" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>fob</t>
+          <t>F.O.B.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>45 dias</t>
+          <t>21 dias</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>13-07-26</t>
+          <t>14/07/2026</t>
         </is>
       </c>
     </row>
@@ -1018,189 +1060,1968 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verniz UV brilho</t>
+          <t>Papel offset 120g 66x96</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>litro</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Gráfica Suprimentos SA</t>
+          <t>Papelaria Norte</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>93.5</v>
+        <v>198</v>
       </c>
       <c r="G17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>C.I.F.</t>
+          <t>CIF</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>à vista (3% desc.)</t>
+          <t>28 dias</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>13/07/2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Chapa CTP violeta 745x605</t>
+          <t>Papel offset 120g 66x96</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Papelaria Norte</t>
+          <t>Insumos Delta</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>41,50</t>
+          <t>191,00</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CIF</t>
+          <t>fob</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>28 dias</t>
+          <t>45 dias</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>13/07/2026</t>
+          <t>13-07-26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Chapa CTP violeta 745x605</t>
+          <t>Papel offset 120g 66x96</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>un</t>
+          <t>resma</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Insumos Delta</t>
+          <t>Gráfica Suprimentos SA</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>39.8</v>
+        <v>194.5</v>
       </c>
       <c r="G19" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>fob</t>
+          <t>C.I.F.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>45 dias</t>
+          <t>à vista (3% desc.)</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>13-07-26</t>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Papel offset 120g 66x96</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>35</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>189</v>
+      </c>
+      <c r="G20" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
         <v>5</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cartão duplex 250g 70x100</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>60</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>412,00</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cartão duplex 250g 70x100</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>60</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>398</v>
+      </c>
+      <c r="G22" t="n">
+        <v>12</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>5</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cartão duplex 250g 70x100</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>60</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>405</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Cartão duplex 250g 70x100</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>60</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>401,50</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>3</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cartão triplex 300g 70x100</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>25</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>487</v>
+      </c>
+      <c r="G25" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>6</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cartão triplex 300g 70x100</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>469</v>
+      </c>
+      <c r="G26" t="n">
+        <v>12</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>6</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Cartão triplex 300g 70x100</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>25</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cartão triplex 300g 70x100</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>resma</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>25</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>474</v>
+      </c>
+      <c r="G28" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>7</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tinta escala cyan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>18</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>148</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>7</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Tinta escala cyan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>18</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>139,00</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>12</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tinta escala cyan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>18</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>142.5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Tinta escala cyan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>18</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>141</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>8</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Tinta escala magenta</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>18</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>151</v>
+      </c>
+      <c r="G34" t="n">
+        <v>4</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>8</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Tinta escala magenta</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>18</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>142</v>
+      </c>
+      <c r="G35" t="n">
+        <v>12</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>8</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Tinta escala magenta</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>18</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>145,00</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Tinta escala magenta</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>18</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>143.5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>9</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Tinta escala amarela</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>18</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>146</v>
+      </c>
+      <c r="G38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>9</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Tinta escala amarela</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>18</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>137,50</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>12</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>9</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Tinta escala amarela</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>18</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>140</v>
+      </c>
+      <c r="G40" t="n">
+        <v>6</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>9</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Tinta escala amarela</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>18</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>10</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Tinta escala preta</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>30</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>132,00</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>10</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Tinta escala preta</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>30</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>124</v>
+      </c>
+      <c r="G43" t="n">
+        <v>12</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>10</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Tinta escala preta</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>30</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="G44" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>10</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Tinta escala preta</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>30</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>126,00</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>3</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>11</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Verniz UV brilho</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>25</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>96</v>
+      </c>
+      <c r="G46" t="n">
+        <v>4</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>11</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Verniz UV brilho</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>25</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>91</v>
+      </c>
+      <c r="G47" t="n">
+        <v>12</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>11</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Verniz UV brilho</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>25</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>93,50</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>6</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>11</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Verniz UV brilho</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>25</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>92</v>
+      </c>
+      <c r="G49" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>12</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Verniz acrílico fosco</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>15</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>88.5</v>
+      </c>
+      <c r="G50" t="n">
+        <v>4</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>12</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Verniz acrílico fosco</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>15</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>84,00</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>12</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>12</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Verniz acrílico fosco</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>15</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>6</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>12</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Verniz acrílico fosco</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>litro</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>15</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="G53" t="n">
+        <v>3</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>13</v>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>Chapa CTP violeta 745x605</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>un</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D54" t="n">
         <v>60</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>41,50</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>4</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>13</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Chapa CTP violeta 745x605</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>60</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="G55" t="n">
+        <v>12</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>13</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Chapa CTP violeta 745x605</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>60</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>Gráfica Suprimentos SA</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F56" t="n">
         <v>40.2</v>
       </c>
-      <c r="G20" t="n">
+      <c r="G56" t="n">
         <v>6</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>C.I.F.</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>à vista (3% desc.)</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Frete FOB Insumos Delta: R$ 890,00 (não incluso no valor unitário)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="n">
+        <v>13</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Chapa CTP violeta 745x605</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>cx c/ 10</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>60</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>398,00</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>3</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>14</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Chapa CTP térmica 1030x790</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>45</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Papelaria Norte</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>68</v>
+      </c>
+      <c r="G58" t="n">
+        <v>4</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>CIF</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>28 dias</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>14</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Chapa CTP térmica 1030x790</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>45</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Insumos Delta</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="G59" t="n">
+        <v>12</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>fob</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>45 dias</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>13-07-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>14</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Chapa CTP térmica 1030x790</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>45</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Gráfica Suprimentos SA</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>66,00</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>6</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>C.I.F.</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>à vista (3% desc.)</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Chapa CTP térmica 1030x790</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>un</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>45</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Distribuidora Cearapel</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>3</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>F.O.B.</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>21 dias</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Frete FOB por conta da Aurora: Insumos Delta R$ 890,00 · Distribuidora Cearapel R$ 1.240,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>Produção da OS 2481 entra em máquina em 22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Cotações válidas por 5 dias corridos a partir da data de envio</t>
         </is>
       </c>
     </row>

</xml_diff>